<commit_message>
Created by Mena Adel
</commit_message>
<xml_diff>
--- a/Unified_Form_Formatted.xlsx
+++ b/Unified_Form_Formatted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOQ\source\repos\FUTURE_POP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c86ad4d7f8c545c5/Desktop/My Folders/NTI-Python/Project/Future-Pop-2.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{F2E9E9C0-7BAF-4B7B-B96A-53C66FA09863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2684FAA0-10CB-4600-BB66-BF13D42CE0D9}"/>
+    <workbookView minimized="1" xWindow="3168" yWindow="3168" windowWidth="17280" windowHeight="8880" xr2:uid="{2684FAA0-10CB-4600-BB66-BF13D42CE0D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -619,13 +619,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA1882D5-9167-46E8-A1E7-F13E09BAEE2E}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="9" width="13.7109375" customWidth="1"/>
-    <col min="10" max="15" width="12.28515625" customWidth="1"/>
+    <col min="1" max="9" width="13.6640625" customWidth="1"/>
+    <col min="10" max="15" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" customHeight="1">
+    <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -654,7 +654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="21" customHeight="1">
+    <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -683,7 +683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="20.45" customHeight="1">
+    <row r="3" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -712,7 +712,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="20.45" customHeight="1">
+    <row r="4" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -741,7 +741,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="20.45" customHeight="1">
+    <row r="5" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -770,7 +770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="20.45" customHeight="1">
+    <row r="6" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -799,7 +799,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="20.45" customHeight="1">
+    <row r="7" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
@@ -828,7 +828,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="20.45" customHeight="1">
+    <row r="8" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -857,7 +857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="20.45" customHeight="1">
+    <row r="9" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -886,7 +886,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="20.45" customHeight="1">
+    <row r="10" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>19</v>
       </c>
@@ -915,7 +915,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="20.45" customHeight="1">
+    <row r="11" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -944,7 +944,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="20.45" customHeight="1">
+    <row r="12" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -973,7 +973,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="20.45" customHeight="1">
+    <row r="13" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>23</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="20.45" customHeight="1">
+    <row r="14" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="20.45" customHeight="1">
+    <row r="15" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="20.45" customHeight="1">
+    <row r="16" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>28</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="20.45" customHeight="1">
+    <row r="17" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="20.45" customHeight="1">
+    <row r="18" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="20.45" customHeight="1">
+    <row r="19" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>31</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="20.45" customHeight="1">
+    <row r="20" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="20.45" customHeight="1">
+    <row r="21" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>34</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="20.45" customHeight="1">
+    <row r="22" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>35</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="20.45" customHeight="1">
+    <row r="23" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>36</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="20.45" customHeight="1">
+    <row r="24" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>37</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="20.45" customHeight="1">
+    <row r="25" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>40</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="20.45" customHeight="1">
+    <row r="26" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>43</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="20.45" customHeight="1">
+    <row r="27" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>45</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="20.45" customHeight="1">
+    <row r="28" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>47</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="20.45" customHeight="1"/>
+    <row r="29" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I28">
     <sortCondition descending="1" ref="G3:G28"/>
@@ -1455,5 +1455,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD41EB08-BDFF-4D6D-A3B5-316B5365B71B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD41EB08-BDFF-4D6D-A3B5-316B5365B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add fixed version of the Data sheet
</commit_message>
<xml_diff>
--- a/Unified_Form_Formatted.xlsx
+++ b/Unified_Form_Formatted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c86ad4d7f8c545c5/Desktop/My Folders/NTI-Python/Project/Future-Pop-2.0/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOQ\source\repos\FUTURE_POP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2E9E9C0-7BAF-4B7B-B96A-53C66FA09863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{33E0C48A-0F2E-44BD-BC12-A9A849AC774F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3168" yWindow="3168" windowWidth="17280" windowHeight="8880" xr2:uid="{2684FAA0-10CB-4600-BB66-BF13D42CE0D9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2684FAA0-10CB-4600-BB66-BF13D42CE0D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="49">
   <si>
-    <t xml:space="preserve">Governorate </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Capital</t>
+    <t>Governorate</t>
+  </si>
+  <si>
+    <t>Capital</t>
   </si>
   <si>
     <t>Area</t>
@@ -189,7 +189,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -619,13 +619,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA1882D5-9167-46E8-A1E7-F13E09BAEE2E}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="9" width="13.6640625" customWidth="1"/>
-    <col min="10" max="15" width="12.33203125" customWidth="1"/>
+    <col min="1" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="15" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="21" customHeight="1">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -654,7 +654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="21" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -683,7 +683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="20.45" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -712,7 +712,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="20.45" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -741,7 +741,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="20.45" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -770,7 +770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="20.45" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -799,7 +799,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="20.45" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
@@ -828,7 +828,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="20.45" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -857,7 +857,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="20.45" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -886,7 +886,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="20.45" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>19</v>
       </c>
@@ -915,7 +915,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="20.45" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -944,7 +944,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="20.45" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -973,7 +973,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="20.45" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>23</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="20.45" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="20.45" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="20.45" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>28</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="20.45" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="20.45" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="20.45" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>31</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="20.45" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="20.45" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>34</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="20.45" customHeight="1">
       <c r="A22" s="4" t="s">
         <v>35</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="20.45" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>36</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="20.45" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>37</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="20.45" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>40</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="20.45" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>43</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="20.45" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>45</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="20.45" customHeight="1">
       <c r="A28" s="4" t="s">
         <v>47</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:9" ht="20.45" customHeight="1"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I28">
     <sortCondition descending="1" ref="G3:G28"/>
@@ -1455,9 +1455,5 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD41EB08-BDFF-4D6D-A3B5-316B5365B71B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD41EB08-BDFF-4D6D-A3B5-316B5365B71B}"/>
 </file>
</xml_diff>